<commit_message>
Changes to be committed: 	modified:   apps/api/src/students/import/student-import.service.ts 	modified:   apps/web/app/(app)/change-requests/page.tsx 	modified:   apps/web/app/(app)/me/change-requests/page.tsx 	modified:   apps/web/app/(app)/me/profile/page.tsx 	modified:   apps/web/app/(app)/students/[id]/page.tsx 	modified:   apps/web/app/(app)/students/import/page.tsx 	modified:   apps/web/app/(app)/students/new/page.tsx 	modified:   apps/web/app/activate/page.tsx 	new file:   apps/web/lib/dates.ts 	modified:   apps/web/public/templates/student-import-template.csv 	modified:   apps/web/public/templates/student-import-template.xlsx 	modified:   docs/28-DEV-SETUP.md 	modified:   docs/templates/student-import-template.csv 	modified:   docs/templates/student-import-template.xlsx
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/student-import-template.xlsx
+++ b/apps/web/public/templates/student-import-template.xlsx
@@ -76,7 +76,7 @@
     <t>Ngozi</t>
   </si>
   <si>
-    <t>2005-01-02</t>
+    <t>02/01/2005</t>
   </si>
   <si>
     <t>FEMALE</t>
@@ -121,7 +121,7 @@
     <t/>
   </si>
   <si>
-    <t>2004-11-15</t>
+    <t>15/11/2004</t>
   </si>
   <si>
     <t>MALE</t>
@@ -145,7 +145,7 @@
     <t>Bisi</t>
   </si>
   <si>
-    <t>2005-06-30</t>
+    <t>30/06/2005</t>
   </si>
   <si>
     <t>MTH</t>
@@ -169,7 +169,7 @@
     <t>Yusuf</t>
   </si>
   <si>
-    <t>2003-09-09</t>
+    <t>09/09/2003</t>
   </si>
   <si>
     <t>ENG</t>
@@ -838,6 +838,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>